<commit_message>
correccion de errores en la importacion de vocerias
</commit_message>
<xml_diff>
--- a/assets/templates/plantilla_importacion_voceria.xlsx
+++ b/assets/templates/plantilla_importacion_voceria.xlsx
@@ -15,7 +15,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -125,7 +127,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -139,6 +141,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -507,7 +515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R32"/>
+  <dimension ref="A1:R12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="8.28515625" customWidth="1" style="1" min="1" max="1"/>
@@ -658,14 +666,14 @@
       <c r="H3" s="3" t="n"/>
       <c r="I3" s="3" t="n"/>
       <c r="J3" s="3" t="n"/>
-      <c r="K3" s="3" t="n"/>
+      <c r="K3" s="8" t="n"/>
       <c r="L3" s="3" t="n"/>
-      <c r="M3" s="3" t="n"/>
+      <c r="M3" s="7" t="n"/>
       <c r="N3" s="3" t="n"/>
       <c r="O3" s="3" t="n"/>
       <c r="P3" s="3" t="n"/>
       <c r="Q3" s="3" t="n"/>
-      <c r="R3" s="3" t="n"/>
+      <c r="R3" s="7" t="n"/>
     </row>
     <row r="4" ht="25.5" customHeight="1" s="1">
       <c r="A4" s="3" t="n">
@@ -680,14 +688,14 @@
       <c r="H4" s="3" t="n"/>
       <c r="I4" s="3" t="n"/>
       <c r="J4" s="3" t="n"/>
-      <c r="K4" s="3" t="n"/>
+      <c r="K4" s="8" t="n"/>
       <c r="L4" s="3" t="n"/>
-      <c r="M4" s="3" t="n"/>
+      <c r="M4" s="7" t="n"/>
       <c r="N4" s="3" t="n"/>
       <c r="O4" s="3" t="n"/>
       <c r="P4" s="3" t="n"/>
       <c r="Q4" s="3" t="n"/>
-      <c r="R4" s="3" t="n"/>
+      <c r="R4" s="7" t="n"/>
     </row>
     <row r="5" ht="25.5" customHeight="1" s="1">
       <c r="A5" s="3" t="n">
@@ -702,14 +710,14 @@
       <c r="H5" s="3" t="n"/>
       <c r="I5" s="3" t="n"/>
       <c r="J5" s="3" t="n"/>
-      <c r="K5" s="3" t="n"/>
+      <c r="K5" s="8" t="n"/>
       <c r="L5" s="3" t="n"/>
-      <c r="M5" s="3" t="n"/>
+      <c r="M5" s="7" t="n"/>
       <c r="N5" s="3" t="n"/>
       <c r="O5" s="3" t="n"/>
       <c r="P5" s="3" t="n"/>
       <c r="Q5" s="3" t="n"/>
-      <c r="R5" s="3" t="n"/>
+      <c r="R5" s="7" t="n"/>
     </row>
     <row r="6" ht="25.5" customHeight="1" s="1">
       <c r="A6" s="3" t="n">
@@ -724,14 +732,14 @@
       <c r="H6" s="3" t="n"/>
       <c r="I6" s="3" t="n"/>
       <c r="J6" s="3" t="n"/>
-      <c r="K6" s="3" t="n"/>
+      <c r="K6" s="8" t="n"/>
       <c r="L6" s="3" t="n"/>
-      <c r="M6" s="3" t="n"/>
+      <c r="M6" s="7" t="n"/>
       <c r="N6" s="3" t="n"/>
       <c r="O6" s="3" t="n"/>
       <c r="P6" s="3" t="n"/>
       <c r="Q6" s="3" t="n"/>
-      <c r="R6" s="3" t="n"/>
+      <c r="R6" s="7" t="n"/>
     </row>
     <row r="7" ht="25.5" customHeight="1" s="1">
       <c r="A7" s="3" t="n">
@@ -746,14 +754,14 @@
       <c r="H7" s="3" t="n"/>
       <c r="I7" s="3" t="n"/>
       <c r="J7" s="3" t="n"/>
-      <c r="K7" s="3" t="n"/>
+      <c r="K7" s="8" t="n"/>
       <c r="L7" s="3" t="n"/>
-      <c r="M7" s="3" t="n"/>
+      <c r="M7" s="7" t="n"/>
       <c r="N7" s="3" t="n"/>
       <c r="O7" s="3" t="n"/>
       <c r="P7" s="3" t="n"/>
       <c r="Q7" s="3" t="n"/>
-      <c r="R7" s="3" t="n"/>
+      <c r="R7" s="7" t="n"/>
     </row>
     <row r="8" ht="25.5" customHeight="1" s="1">
       <c r="A8" s="3" t="n">
@@ -768,14 +776,14 @@
       <c r="H8" s="3" t="n"/>
       <c r="I8" s="3" t="n"/>
       <c r="J8" s="3" t="n"/>
-      <c r="K8" s="3" t="n"/>
+      <c r="K8" s="8" t="n"/>
       <c r="L8" s="3" t="n"/>
-      <c r="M8" s="3" t="n"/>
+      <c r="M8" s="7" t="n"/>
       <c r="N8" s="3" t="n"/>
       <c r="O8" s="3" t="n"/>
       <c r="P8" s="3" t="n"/>
       <c r="Q8" s="3" t="n"/>
-      <c r="R8" s="3" t="n"/>
+      <c r="R8" s="7" t="n"/>
     </row>
     <row r="9" ht="25.5" customHeight="1" s="1">
       <c r="A9" s="3" t="n">
@@ -790,14 +798,14 @@
       <c r="H9" s="3" t="n"/>
       <c r="I9" s="3" t="n"/>
       <c r="J9" s="3" t="n"/>
-      <c r="K9" s="3" t="n"/>
+      <c r="K9" s="8" t="n"/>
       <c r="L9" s="3" t="n"/>
-      <c r="M9" s="3" t="n"/>
+      <c r="M9" s="7" t="n"/>
       <c r="N9" s="3" t="n"/>
       <c r="O9" s="3" t="n"/>
       <c r="P9" s="3" t="n"/>
       <c r="Q9" s="3" t="n"/>
-      <c r="R9" s="3" t="n"/>
+      <c r="R9" s="7" t="n"/>
     </row>
     <row r="10" ht="25.5" customHeight="1" s="1">
       <c r="A10" s="3" t="n">
@@ -812,14 +820,14 @@
       <c r="H10" s="3" t="n"/>
       <c r="I10" s="3" t="n"/>
       <c r="J10" s="3" t="n"/>
-      <c r="K10" s="3" t="n"/>
+      <c r="K10" s="8" t="n"/>
       <c r="L10" s="3" t="n"/>
-      <c r="M10" s="3" t="n"/>
+      <c r="M10" s="7" t="n"/>
       <c r="N10" s="3" t="n"/>
       <c r="O10" s="3" t="n"/>
       <c r="P10" s="3" t="n"/>
       <c r="Q10" s="3" t="n"/>
-      <c r="R10" s="3" t="n"/>
+      <c r="R10" s="7" t="n"/>
     </row>
     <row r="11" ht="25.5" customHeight="1" s="1">
       <c r="A11" s="3" t="n">
@@ -834,14 +842,14 @@
       <c r="H11" s="3" t="n"/>
       <c r="I11" s="3" t="n"/>
       <c r="J11" s="3" t="n"/>
-      <c r="K11" s="3" t="n"/>
+      <c r="K11" s="8" t="n"/>
       <c r="L11" s="3" t="n"/>
-      <c r="M11" s="3" t="n"/>
+      <c r="M11" s="7" t="n"/>
       <c r="N11" s="3" t="n"/>
       <c r="O11" s="3" t="n"/>
       <c r="P11" s="3" t="n"/>
       <c r="Q11" s="3" t="n"/>
-      <c r="R11" s="3" t="n"/>
+      <c r="R11" s="7" t="n"/>
     </row>
     <row r="12" ht="25.5" customHeight="1" s="1">
       <c r="A12" s="3" t="n">
@@ -856,460 +864,40 @@
       <c r="H12" s="3" t="n"/>
       <c r="I12" s="3" t="n"/>
       <c r="J12" s="3" t="n"/>
-      <c r="K12" s="3" t="n"/>
+      <c r="K12" s="8" t="n"/>
       <c r="L12" s="3" t="n"/>
-      <c r="M12" s="3" t="n"/>
+      <c r="M12" s="7" t="n"/>
       <c r="N12" s="3" t="n"/>
       <c r="O12" s="3" t="n"/>
       <c r="P12" s="3" t="n"/>
       <c r="Q12" s="3" t="n"/>
-      <c r="R12" s="3" t="n"/>
-    </row>
-    <row r="13" ht="25.5" customHeight="1" s="1">
-      <c r="A13" s="3" t="n">
-        <v>11</v>
-      </c>
-      <c r="B13" s="3" t="n"/>
-      <c r="C13" s="3" t="n"/>
-      <c r="D13" s="3" t="n"/>
-      <c r="E13" s="3" t="n"/>
-      <c r="F13" s="3" t="n"/>
-      <c r="G13" s="3" t="n"/>
-      <c r="H13" s="3" t="n"/>
-      <c r="I13" s="3" t="n"/>
-      <c r="J13" s="3" t="n"/>
-      <c r="K13" s="3" t="n"/>
-      <c r="L13" s="3" t="n"/>
-      <c r="M13" s="3" t="n"/>
-      <c r="N13" s="3" t="n"/>
-      <c r="O13" s="3" t="n"/>
-      <c r="P13" s="3" t="n"/>
-      <c r="Q13" s="3" t="n"/>
-      <c r="R13" s="3" t="n"/>
-    </row>
-    <row r="14" ht="25.5" customHeight="1" s="1">
-      <c r="A14" s="3" t="n">
-        <v>12</v>
-      </c>
-      <c r="B14" s="3" t="n"/>
-      <c r="C14" s="3" t="n"/>
-      <c r="D14" s="3" t="n"/>
-      <c r="E14" s="3" t="n"/>
-      <c r="F14" s="3" t="n"/>
-      <c r="G14" s="3" t="n"/>
-      <c r="H14" s="3" t="n"/>
-      <c r="I14" s="3" t="n"/>
-      <c r="J14" s="3" t="n"/>
-      <c r="K14" s="3" t="n"/>
-      <c r="L14" s="3" t="n"/>
-      <c r="M14" s="3" t="n"/>
-      <c r="N14" s="3" t="n"/>
-      <c r="O14" s="3" t="n"/>
-      <c r="P14" s="3" t="n"/>
-      <c r="Q14" s="3" t="n"/>
-      <c r="R14" s="3" t="n"/>
-    </row>
-    <row r="15" ht="25.5" customHeight="1" s="1">
-      <c r="A15" s="3" t="n">
-        <v>13</v>
-      </c>
-      <c r="B15" s="3" t="n"/>
-      <c r="C15" s="3" t="n"/>
-      <c r="D15" s="3" t="n"/>
-      <c r="E15" s="3" t="n"/>
-      <c r="F15" s="3" t="n"/>
-      <c r="G15" s="3" t="n"/>
-      <c r="H15" s="3" t="n"/>
-      <c r="I15" s="3" t="n"/>
-      <c r="J15" s="3" t="n"/>
-      <c r="K15" s="3" t="n"/>
-      <c r="L15" s="3" t="n"/>
-      <c r="M15" s="3" t="n"/>
-      <c r="N15" s="3" t="n"/>
-      <c r="O15" s="3" t="n"/>
-      <c r="P15" s="3" t="n"/>
-      <c r="Q15" s="3" t="n"/>
-      <c r="R15" s="3" t="n"/>
-    </row>
-    <row r="16" ht="25.5" customHeight="1" s="1">
-      <c r="A16" s="3" t="n">
-        <v>14</v>
-      </c>
-      <c r="B16" s="3" t="n"/>
-      <c r="C16" s="3" t="n"/>
-      <c r="D16" s="3" t="n"/>
-      <c r="E16" s="3" t="n"/>
-      <c r="F16" s="3" t="n"/>
-      <c r="G16" s="3" t="n"/>
-      <c r="H16" s="3" t="n"/>
-      <c r="I16" s="3" t="n"/>
-      <c r="J16" s="3" t="n"/>
-      <c r="K16" s="3" t="n"/>
-      <c r="L16" s="3" t="n"/>
-      <c r="M16" s="3" t="n"/>
-      <c r="N16" s="3" t="n"/>
-      <c r="O16" s="3" t="n"/>
-      <c r="P16" s="3" t="n"/>
-      <c r="Q16" s="3" t="n"/>
-      <c r="R16" s="3" t="n"/>
-    </row>
-    <row r="17" ht="25.5" customHeight="1" s="1">
-      <c r="A17" s="3" t="n">
-        <v>15</v>
-      </c>
-      <c r="B17" s="3" t="n"/>
-      <c r="C17" s="3" t="n"/>
-      <c r="D17" s="3" t="n"/>
-      <c r="E17" s="3" t="n"/>
-      <c r="F17" s="3" t="n"/>
-      <c r="G17" s="3" t="n"/>
-      <c r="H17" s="3" t="n"/>
-      <c r="I17" s="3" t="n"/>
-      <c r="J17" s="3" t="n"/>
-      <c r="K17" s="3" t="n"/>
-      <c r="L17" s="3" t="n"/>
-      <c r="M17" s="3" t="n"/>
-      <c r="N17" s="3" t="n"/>
-      <c r="O17" s="3" t="n"/>
-      <c r="P17" s="3" t="n"/>
-      <c r="Q17" s="3" t="n"/>
-      <c r="R17" s="3" t="n"/>
-    </row>
-    <row r="18" ht="25.5" customHeight="1" s="1">
-      <c r="A18" s="3" t="n">
-        <v>16</v>
-      </c>
-      <c r="B18" s="3" t="n"/>
-      <c r="C18" s="3" t="n"/>
-      <c r="D18" s="3" t="n"/>
-      <c r="E18" s="3" t="n"/>
-      <c r="F18" s="3" t="n"/>
-      <c r="G18" s="3" t="n"/>
-      <c r="H18" s="3" t="n"/>
-      <c r="I18" s="3" t="n"/>
-      <c r="J18" s="3" t="n"/>
-      <c r="K18" s="3" t="n"/>
-      <c r="L18" s="3" t="n"/>
-      <c r="M18" s="3" t="n"/>
-      <c r="N18" s="3" t="n"/>
-      <c r="O18" s="3" t="n"/>
-      <c r="P18" s="3" t="n"/>
-      <c r="Q18" s="3" t="n"/>
-      <c r="R18" s="3" t="n"/>
-    </row>
-    <row r="19" ht="25.5" customHeight="1" s="1">
-      <c r="A19" s="3" t="n">
-        <v>17</v>
-      </c>
-      <c r="B19" s="3" t="n"/>
-      <c r="C19" s="3" t="n"/>
-      <c r="D19" s="3" t="n"/>
-      <c r="E19" s="3" t="n"/>
-      <c r="F19" s="3" t="n"/>
-      <c r="G19" s="3" t="n"/>
-      <c r="H19" s="3" t="n"/>
-      <c r="I19" s="3" t="n"/>
-      <c r="J19" s="3" t="n"/>
-      <c r="K19" s="3" t="n"/>
-      <c r="L19" s="3" t="n"/>
-      <c r="M19" s="3" t="n"/>
-      <c r="N19" s="3" t="n"/>
-      <c r="O19" s="3" t="n"/>
-      <c r="P19" s="3" t="n"/>
-      <c r="Q19" s="3" t="n"/>
-      <c r="R19" s="3" t="n"/>
-    </row>
-    <row r="20" ht="25.5" customHeight="1" s="1">
-      <c r="A20" s="3" t="n">
-        <v>18</v>
-      </c>
-      <c r="B20" s="3" t="n"/>
-      <c r="C20" s="3" t="n"/>
-      <c r="D20" s="3" t="n"/>
-      <c r="E20" s="3" t="n"/>
-      <c r="F20" s="3" t="n"/>
-      <c r="G20" s="3" t="n"/>
-      <c r="H20" s="3" t="n"/>
-      <c r="I20" s="3" t="n"/>
-      <c r="J20" s="3" t="n"/>
-      <c r="K20" s="3" t="n"/>
-      <c r="L20" s="3" t="n"/>
-      <c r="M20" s="3" t="n"/>
-      <c r="N20" s="3" t="n"/>
-      <c r="O20" s="3" t="n"/>
-      <c r="P20" s="3" t="n"/>
-      <c r="Q20" s="3" t="n"/>
-      <c r="R20" s="3" t="n"/>
-    </row>
-    <row r="21" ht="25.5" customHeight="1" s="1">
-      <c r="A21" s="3" t="n">
-        <v>19</v>
-      </c>
-      <c r="B21" s="3" t="n"/>
-      <c r="C21" s="3" t="n"/>
-      <c r="D21" s="3" t="n"/>
-      <c r="E21" s="3" t="n"/>
-      <c r="F21" s="3" t="n"/>
-      <c r="G21" s="3" t="n"/>
-      <c r="H21" s="3" t="n"/>
-      <c r="I21" s="3" t="n"/>
-      <c r="J21" s="3" t="n"/>
-      <c r="K21" s="3" t="n"/>
-      <c r="L21" s="3" t="n"/>
-      <c r="M21" s="3" t="n"/>
-      <c r="N21" s="3" t="n"/>
-      <c r="O21" s="3" t="n"/>
-      <c r="P21" s="3" t="n"/>
-      <c r="Q21" s="3" t="n"/>
-      <c r="R21" s="3" t="n"/>
-    </row>
-    <row r="22" ht="25.5" customHeight="1" s="1">
-      <c r="A22" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="B22" s="3" t="n"/>
-      <c r="C22" s="3" t="n"/>
-      <c r="D22" s="3" t="n"/>
-      <c r="E22" s="3" t="n"/>
-      <c r="F22" s="3" t="n"/>
-      <c r="G22" s="3" t="n"/>
-      <c r="H22" s="3" t="n"/>
-      <c r="I22" s="3" t="n"/>
-      <c r="J22" s="3" t="n"/>
-      <c r="K22" s="3" t="n"/>
-      <c r="L22" s="3" t="n"/>
-      <c r="M22" s="3" t="n"/>
-      <c r="N22" s="3" t="n"/>
-      <c r="O22" s="3" t="n"/>
-      <c r="P22" s="3" t="n"/>
-      <c r="Q22" s="3" t="n"/>
-      <c r="R22" s="3" t="n"/>
-    </row>
-    <row r="23" ht="25.5" customHeight="1" s="1">
-      <c r="A23" s="3" t="n">
-        <v>21</v>
-      </c>
-      <c r="B23" s="3" t="n"/>
-      <c r="C23" s="3" t="n"/>
-      <c r="D23" s="3" t="n"/>
-      <c r="E23" s="3" t="n"/>
-      <c r="F23" s="3" t="n"/>
-      <c r="G23" s="3" t="n"/>
-      <c r="H23" s="3" t="n"/>
-      <c r="I23" s="3" t="n"/>
-      <c r="J23" s="3" t="n"/>
-      <c r="K23" s="3" t="n"/>
-      <c r="L23" s="3" t="n"/>
-      <c r="M23" s="3" t="n"/>
-      <c r="N23" s="3" t="n"/>
-      <c r="O23" s="3" t="n"/>
-      <c r="P23" s="3" t="n"/>
-      <c r="Q23" s="3" t="n"/>
-      <c r="R23" s="3" t="n"/>
-    </row>
-    <row r="24" ht="25.5" customHeight="1" s="1">
-      <c r="A24" s="3" t="n">
-        <v>22</v>
-      </c>
-      <c r="B24" s="3" t="n"/>
-      <c r="C24" s="3" t="n"/>
-      <c r="D24" s="3" t="n"/>
-      <c r="E24" s="3" t="n"/>
-      <c r="F24" s="3" t="n"/>
-      <c r="G24" s="3" t="n"/>
-      <c r="H24" s="3" t="n"/>
-      <c r="I24" s="3" t="n"/>
-      <c r="J24" s="3" t="n"/>
-      <c r="K24" s="3" t="n"/>
-      <c r="L24" s="3" t="n"/>
-      <c r="M24" s="3" t="n"/>
-      <c r="N24" s="3" t="n"/>
-      <c r="O24" s="3" t="n"/>
-      <c r="P24" s="3" t="n"/>
-      <c r="Q24" s="3" t="n"/>
-      <c r="R24" s="3" t="n"/>
-    </row>
-    <row r="25" ht="25.5" customHeight="1" s="1">
-      <c r="A25" s="3" t="n">
-        <v>23</v>
-      </c>
-      <c r="B25" s="3" t="n"/>
-      <c r="C25" s="3" t="n"/>
-      <c r="D25" s="3" t="n"/>
-      <c r="E25" s="3" t="n"/>
-      <c r="F25" s="3" t="n"/>
-      <c r="G25" s="3" t="n"/>
-      <c r="H25" s="3" t="n"/>
-      <c r="I25" s="3" t="n"/>
-      <c r="J25" s="3" t="n"/>
-      <c r="K25" s="3" t="n"/>
-      <c r="L25" s="3" t="n"/>
-      <c r="M25" s="3" t="n"/>
-      <c r="N25" s="3" t="n"/>
-      <c r="O25" s="3" t="n"/>
-      <c r="P25" s="3" t="n"/>
-      <c r="Q25" s="3" t="n"/>
-      <c r="R25" s="3" t="n"/>
-    </row>
-    <row r="26" ht="25.5" customHeight="1" s="1">
-      <c r="A26" s="3" t="n">
-        <v>24</v>
-      </c>
-      <c r="B26" s="3" t="n"/>
-      <c r="C26" s="3" t="n"/>
-      <c r="D26" s="3" t="n"/>
-      <c r="E26" s="3" t="n"/>
-      <c r="F26" s="3" t="n"/>
-      <c r="G26" s="3" t="n"/>
-      <c r="H26" s="3" t="n"/>
-      <c r="I26" s="3" t="n"/>
-      <c r="J26" s="3" t="n"/>
-      <c r="K26" s="3" t="n"/>
-      <c r="L26" s="3" t="n"/>
-      <c r="M26" s="3" t="n"/>
-      <c r="N26" s="3" t="n"/>
-      <c r="O26" s="3" t="n"/>
-      <c r="P26" s="3" t="n"/>
-      <c r="Q26" s="3" t="n"/>
-      <c r="R26" s="3" t="n"/>
-    </row>
-    <row r="27" ht="25.5" customHeight="1" s="1">
-      <c r="A27" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="B27" s="3" t="n"/>
-      <c r="C27" s="3" t="n"/>
-      <c r="D27" s="3" t="n"/>
-      <c r="E27" s="3" t="n"/>
-      <c r="F27" s="3" t="n"/>
-      <c r="G27" s="3" t="n"/>
-      <c r="H27" s="3" t="n"/>
-      <c r="I27" s="3" t="n"/>
-      <c r="J27" s="3" t="n"/>
-      <c r="K27" s="3" t="n"/>
-      <c r="L27" s="3" t="n"/>
-      <c r="M27" s="3" t="n"/>
-      <c r="N27" s="3" t="n"/>
-      <c r="O27" s="3" t="n"/>
-      <c r="P27" s="3" t="n"/>
-      <c r="Q27" s="3" t="n"/>
-      <c r="R27" s="3" t="n"/>
-    </row>
-    <row r="28" ht="25.5" customHeight="1" s="1">
-      <c r="A28" s="3" t="n">
-        <v>26</v>
-      </c>
-      <c r="B28" s="3" t="n"/>
-      <c r="C28" s="3" t="n"/>
-      <c r="D28" s="3" t="n"/>
-      <c r="E28" s="3" t="n"/>
-      <c r="F28" s="3" t="n"/>
-      <c r="G28" s="3" t="n"/>
-      <c r="H28" s="3" t="n"/>
-      <c r="I28" s="3" t="n"/>
-      <c r="J28" s="3" t="n"/>
-      <c r="K28" s="3" t="n"/>
-      <c r="L28" s="3" t="n"/>
-      <c r="M28" s="3" t="n"/>
-      <c r="N28" s="3" t="n"/>
-      <c r="O28" s="3" t="n"/>
-      <c r="P28" s="3" t="n"/>
-      <c r="Q28" s="3" t="n"/>
-      <c r="R28" s="3" t="n"/>
-    </row>
-    <row r="29" ht="25.5" customHeight="1" s="1">
-      <c r="A29" s="3" t="n">
-        <v>27</v>
-      </c>
-      <c r="B29" s="3" t="n"/>
-      <c r="C29" s="3" t="n"/>
-      <c r="D29" s="3" t="n"/>
-      <c r="E29" s="3" t="n"/>
-      <c r="F29" s="3" t="n"/>
-      <c r="G29" s="3" t="n"/>
-      <c r="H29" s="3" t="n"/>
-      <c r="I29" s="3" t="n"/>
-      <c r="J29" s="3" t="n"/>
-      <c r="K29" s="3" t="n"/>
-      <c r="L29" s="3" t="n"/>
-      <c r="M29" s="3" t="n"/>
-      <c r="N29" s="3" t="n"/>
-      <c r="O29" s="3" t="n"/>
-      <c r="P29" s="3" t="n"/>
-      <c r="Q29" s="3" t="n"/>
-      <c r="R29" s="3" t="n"/>
-    </row>
-    <row r="30" ht="25.5" customHeight="1" s="1">
-      <c r="A30" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="B30" s="3" t="n"/>
-      <c r="C30" s="3" t="n"/>
-      <c r="D30" s="3" t="n"/>
-      <c r="E30" s="3" t="n"/>
-      <c r="F30" s="3" t="n"/>
-      <c r="G30" s="3" t="n"/>
-      <c r="H30" s="3" t="n"/>
-      <c r="I30" s="3" t="n"/>
-      <c r="J30" s="3" t="n"/>
-      <c r="K30" s="3" t="n"/>
-      <c r="L30" s="3" t="n"/>
-      <c r="M30" s="3" t="n"/>
-      <c r="N30" s="3" t="n"/>
-      <c r="O30" s="3" t="n"/>
-      <c r="P30" s="3" t="n"/>
-      <c r="Q30" s="3" t="n"/>
-      <c r="R30" s="3" t="n"/>
-    </row>
-    <row r="31" ht="25.5" customHeight="1" s="1">
-      <c r="A31" s="3" t="n">
-        <v>29</v>
-      </c>
-      <c r="B31" s="3" t="n"/>
-      <c r="C31" s="3" t="n"/>
-      <c r="D31" s="3" t="n"/>
-      <c r="E31" s="3" t="n"/>
-      <c r="F31" s="3" t="n"/>
-      <c r="G31" s="3" t="n"/>
-      <c r="H31" s="3" t="n"/>
-      <c r="I31" s="3" t="n"/>
-      <c r="J31" s="3" t="n"/>
-      <c r="K31" s="3" t="n"/>
-      <c r="L31" s="3" t="n"/>
-      <c r="M31" s="3" t="n"/>
-      <c r="N31" s="3" t="n"/>
-      <c r="O31" s="3" t="n"/>
-      <c r="P31" s="3" t="n"/>
-      <c r="Q31" s="3" t="n"/>
-      <c r="R31" s="3" t="n"/>
-    </row>
-    <row r="32" ht="25.5" customHeight="1" s="1">
-      <c r="A32" s="3" t="n">
-        <v>30</v>
-      </c>
-      <c r="B32" s="3" t="n"/>
-      <c r="C32" s="3" t="n"/>
-      <c r="D32" s="3" t="n"/>
-      <c r="E32" s="3" t="n"/>
-      <c r="F32" s="3" t="n"/>
-      <c r="G32" s="3" t="n"/>
-      <c r="H32" s="3" t="n"/>
-      <c r="I32" s="3" t="n"/>
-      <c r="J32" s="3" t="n"/>
-      <c r="K32" s="3" t="n"/>
-      <c r="L32" s="3" t="n"/>
-      <c r="M32" s="3" t="n"/>
-      <c r="N32" s="3" t="n"/>
-      <c r="O32" s="3" t="n"/>
-      <c r="P32" s="3" t="n"/>
-      <c r="Q32" s="3" t="n"/>
-      <c r="R32" s="3" t="n"/>
-    </row>
+      <c r="R12" s="7" t="n"/>
+    </row>
+    <row r="13" ht="25.5" customHeight="1" s="1"/>
+    <row r="14" ht="25.5" customHeight="1" s="1"/>
+    <row r="15" ht="25.5" customHeight="1" s="1"/>
+    <row r="16" ht="25.5" customHeight="1" s="1"/>
+    <row r="17" ht="25.5" customHeight="1" s="1"/>
+    <row r="18" ht="25.5" customHeight="1" s="1"/>
+    <row r="19" ht="25.5" customHeight="1" s="1"/>
+    <row r="20" ht="25.5" customHeight="1" s="1"/>
+    <row r="21" ht="25.5" customHeight="1" s="1"/>
+    <row r="22" ht="25.5" customHeight="1" s="1"/>
+    <row r="23" ht="25.5" customHeight="1" s="1"/>
+    <row r="24" ht="25.5" customHeight="1" s="1"/>
+    <row r="25" ht="25.5" customHeight="1" s="1"/>
+    <row r="26" ht="25.5" customHeight="1" s="1"/>
+    <row r="27" ht="25.5" customHeight="1" s="1"/>
+    <row r="28" ht="25.5" customHeight="1" s="1"/>
+    <row r="29" ht="25.5" customHeight="1" s="1"/>
+    <row r="30" ht="25.5" customHeight="1" s="1"/>
+    <row r="31" ht="25.5" customHeight="1" s="1"/>
+    <row r="32" ht="25.5" customHeight="1" s="1"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:R1"/>
   </mergeCells>
-  <dataValidations count="5">
+  <dataValidations count="6">
     <dataValidation sqref="B3:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Estado inválido" error="Seleccione un estado válido" promptTitle="Estado" prompt="Seleccione el estado" type="list">
       <formula1>"Táchira"</formula1>
     </dataValidation>
@@ -1325,6 +913,10 @@
     <dataValidation sqref="L3:L1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Vocería inválida" error="Seleccione una vocería válida" promptTitle="Vocería" prompt="Seleccione la vocería" type="list">
       <formula1>"V. CONTRALORÍA,V. DEL ADULTO MAYOR,V. DE ENFERMEDADES CRÓNICAS TRASMISIBLES Y NO TRASMISIBLES,V. DE PERSONAS CON DISCAPACIDAD; ENCAMADOS Y CUIDADORES EN SALUD,V. DE SALUD Y VIDA,V. DE NIÑOS; NIÑAS Y ADOLESCENTES,V. DE LA JUVENTUD EN SALUD,V. DE EDUCACIÓN POPULAR EN SALUD INTERCULTURAL Y ANCESTRAL,V. DE INMUNIZACIONES,V. DE PROYECTOS EN SALUD"</formula1>
     </dataValidation>
+    <dataValidation sqref="M3:M1048576 R3:R1048576" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Fecha no válida" error="Ingrese un valor de fecha válido." promptTitle="Fecha" prompt="Ingrese una fecha válida. Se mostrará como AAAA-MM-DD." type="date" operator="between">
+      <formula1>DATE(1900,1,1)</formula1>
+      <formula2>DATE(9999,12,31)</formula2>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>